<commit_message>
feat: change volume column
</commit_message>
<xml_diff>
--- a/gainers.xlsx
+++ b/gainers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,11 @@
           <t>24h Change</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Volume(24h)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -439,17 +444,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Aerodrome Finance95AERO</t>
+          <t>RaveDAO22RAVE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>$0.455</t>
+          <t>$20.45</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>19.48%</t>
+          <t>21.92%</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>$263,640,007</t>
         </is>
       </c>
     </row>
@@ -459,17 +469,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>币安人生99币安人生</t>
+          <t>Aerodrome Finance95AERO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>$0.3997</t>
+          <t>$0.4565</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>14.58%</t>
+          <t>19.90%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>$45,662,766</t>
         </is>
       </c>
     </row>
@@ -479,17 +494,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RaveDAO22RAVE</t>
+          <t>币安人生99币安人生</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>$19.50</t>
+          <t>$0.3973</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>14.40%</t>
+          <t>14.63%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>$140,503,809</t>
         </is>
       </c>
     </row>
@@ -509,7 +529,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10.84%</t>
+          <t>11.02%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>$27,249,916</t>
         </is>
       </c>
     </row>
@@ -524,12 +549,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>$264.95</t>
+          <t>$266.07</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>10.62%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>$402,912,178</t>
         </is>
       </c>
     </row>
@@ -539,17 +569,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>JUST80JST</t>
+          <t>Ethena54ENA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>$0.06636</t>
+          <t>$0.1175</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>9.89%</t>
+          <t>10.08%</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>$181,482,046</t>
         </is>
       </c>
     </row>
@@ -559,17 +594,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ethena54ENA</t>
+          <t>JUST80JST</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>$0.1176</t>
+          <t>$0.06615</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>9.38%</t>
+          <t>9.29%</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>$55,807,221</t>
         </is>
       </c>
     </row>
@@ -579,17 +619,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>edgeX88EDGE</t>
+          <t>DeXe57DEXE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>$1.30</t>
+          <t>$12.16</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8.46%</t>
+          <t>8.80%</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>$22,591,721</t>
         </is>
       </c>
     </row>
@@ -599,17 +644,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DeXe57DEXE</t>
+          <t>edgeX88EDGE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>$12.15</t>
+          <t>$1.30</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>8.35%</t>
+          <t>8.11%</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>$163,839,829</t>
         </is>
       </c>
     </row>
@@ -629,7 +679,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>7.93%</t>
+          <t>7.99%</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>$36,667,482</t>
         </is>
       </c>
     </row>
@@ -644,12 +699,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>$0.1877</t>
+          <t>$0.1875</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.82%</t>
+          <t>7.96%</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>$46,760,880</t>
         </is>
       </c>
     </row>
@@ -664,12 +724,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>$0.5109</t>
+          <t>$0.5115</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.34%</t>
+          <t>7.80%</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>$43,732,238</t>
         </is>
       </c>
     </row>
@@ -679,17 +744,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Virtuals Protocol84VIRTUAL</t>
+          <t>Venice Token98VVV</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>$0.7761</t>
+          <t>$9.14</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7.08%</t>
+          <t>7.48%</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>$18,638,618</t>
         </is>
       </c>
     </row>
@@ -699,17 +769,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Venice Token98VVV</t>
+          <t>Virtuals Protocol84VIRTUAL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>$9.07</t>
+          <t>$0.7756</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.49%</t>
+          <t>7.18%</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>$131,878,689</t>
         </is>
       </c>
     </row>
@@ -724,12 +799,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$116.71</t>
+          <t>$116.54</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6.13%</t>
+          <t>6.16%</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>$539,567,157</t>
         </is>
       </c>
     </row>
@@ -739,17 +819,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Stellar17XLM</t>
+          <t>Arbitrum67ARB</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$0.1747</t>
+          <t>$0.1308</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>5.56%</t>
+          <t>5.92%</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>$215,481,811</t>
         </is>
       </c>
     </row>
@@ -759,17 +844,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Arbitrum67ARB</t>
+          <t>Stellar17XLM</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>$0.1309</t>
+          <t>$0.1745</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5.42%</t>
+          <t>5.44%</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>$170,548,967</t>
         </is>
       </c>
     </row>
@@ -779,17 +869,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Monad90MON</t>
+          <t>Sky40SKY</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>$0.03697</t>
+          <t>$0.07877</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.10%</t>
+          <t>4.90%</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>$18,685,520</t>
         </is>
       </c>
     </row>
@@ -799,17 +894,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Sky40SKY</t>
+          <t>Monad90MON</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>$0.07887</t>
+          <t>$0.03686</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>5.01%</t>
+          <t>4.89%</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>$105,464,613</t>
         </is>
       </c>
     </row>
@@ -824,12 +924,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>$0.008001</t>
+          <t>$0.007981</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>4.87%</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>$191,776,762</t>
         </is>
       </c>
     </row>
@@ -839,17 +944,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ethereum2ETH</t>
+          <t>Quant62QNT</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>$2,449.17</t>
+          <t>$78.54</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>4.88%</t>
+          <t>4.69%</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>$12,856,050</t>
         </is>
       </c>
     </row>
@@ -859,17 +969,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Quant62QNT</t>
+          <t>Ethereum2ETH</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>$78.68</t>
+          <t>$2,443.98</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4.78%</t>
+          <t>4.51%</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>$25,375,917,895</t>
         </is>
       </c>
     </row>
@@ -884,12 +999,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>$0.1788</t>
+          <t>$0.1785</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>4.67%</t>
+          <t>4.48%</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>$32,751,842</t>
         </is>
       </c>
     </row>
@@ -904,12 +1024,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>$0.6892</t>
+          <t>$0.6888</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4.42%</t>
+          <t>4.39%</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>$51,533,552</t>
         </is>
       </c>
     </row>
@@ -919,17 +1044,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Bitcoin1BTC</t>
+          <t>Pepe46PEPE</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>$77,924.21</t>
+          <t>$0.05405</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.17%</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>$753,685,072</t>
         </is>
       </c>
     </row>
@@ -939,17 +1069,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Pepe46PEPE</t>
+          <t>Bitcoin1BTC</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>$0.054053</t>
+          <t>$77,882.87</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>4.15%</t>
+          <t>4.13%</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>$53,195,207,080</t>
         </is>
       </c>
     </row>
@@ -959,17 +1094,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Solana7SOL</t>
+          <t>Uniswap39UNI</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>$90.24</t>
+          <t>$3.51</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>4.08%</t>
+          <t>3.99%</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>$264,299,084</t>
         </is>
       </c>
     </row>
@@ -979,17 +1119,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GateToken64GT</t>
+          <t>Hedera28HBAR</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>$7.39</t>
+          <t>$0.09227</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4.03%</t>
+          <t>3.98%</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>$131,152,910</t>
         </is>
       </c>
     </row>
@@ -999,17 +1144,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>XRP4XRP</t>
+          <t>Lido DAO101LDO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>$1.49</t>
+          <t>$0.4351</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>3.97%</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>$119,050,022</t>
         </is>
       </c>
     </row>
@@ -1019,17 +1169,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Hedera28HBAR</t>
+          <t>Solana7SOL</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>$0.09235</t>
+          <t>$90.13</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3.94%</t>
+          <t>3.95%</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>$7,643,314,897</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: cleaning data in Gainners and Lossers
</commit_message>
<xml_diff>
--- a/gainers.xlsx
+++ b/gainers.xlsx
@@ -444,22 +444,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>RaveDAO22RAVE</t>
+          <t>RaveDAO21RAVE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>$20.45</t>
+          <t>$20.91</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>21.92%</t>
+          <t>27.46%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>$263,640,007</t>
+          <t>$274,717,861</t>
         </is>
       </c>
     </row>
@@ -469,22 +469,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Aerodrome Finance95AERO</t>
+          <t>Ethena54ENA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>$0.4565</t>
+          <t>$0.1282</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>19.90%</t>
+          <t>14.50%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>$45,662,766</t>
+          <t>$215,822,861</t>
         </is>
       </c>
     </row>
@@ -494,22 +494,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>币安人生99币安人生</t>
+          <t>Aerodrome Finance98AERO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>$0.3973</t>
+          <t>$0.4397</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>14.63%</t>
+          <t>12.13%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>$140,503,809</t>
+          <t>$55,549,454</t>
         </is>
       </c>
     </row>
@@ -519,22 +519,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Morpho65MORPHO</t>
+          <t>DeXe55DEXE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>$1.98</t>
+          <t>$12.29</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>11.02%</t>
+          <t>11.19%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>$27,249,916</t>
+          <t>$23,119,099</t>
         </is>
       </c>
     </row>
@@ -544,22 +544,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bittensor32TAO</t>
+          <t>edgeX86EDGE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>$266.07</t>
+          <t>$1.35</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.62%</t>
+          <t>10.39%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$402,912,178</t>
+          <t>$165,522,350</t>
         </is>
       </c>
     </row>
@@ -569,22 +569,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ethena54ENA</t>
+          <t>Venice Token93VVV</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>$0.1175</t>
+          <t>$9.34</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>$181,482,046</t>
+          <t>$21,763,205</t>
         </is>
       </c>
     </row>
@@ -594,22 +594,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>JUST80JST</t>
+          <t>Morpho67MORPHO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>$0.06615</t>
+          <t>$1.95</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>9.29%</t>
+          <t>8.58%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>$55,807,221</t>
+          <t>$28,951,998</t>
         </is>
       </c>
     </row>
@@ -619,22 +619,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DeXe57DEXE</t>
+          <t>Bittensor32TAO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>$12.16</t>
+          <t>$261.94</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8.80%</t>
+          <t>8.39%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>$22,591,721</t>
+          <t>$415,100,954</t>
         </is>
       </c>
     </row>
@@ -644,22 +644,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>edgeX88EDGE</t>
+          <t>币安人生100币安人生</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>$1.30</t>
+          <t>$0.3666</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>8.11%</t>
+          <t>7.67%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>$163,839,829</t>
+          <t>$143,972,828</t>
         </is>
       </c>
     </row>
@@ -669,22 +669,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Kaspa59KAS</t>
+          <t>JUST79JST</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>$0.0362</t>
+          <t>$0.06753</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>7.99%</t>
+          <t>7.54%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>$36,667,482</t>
+          <t>$51,374,400</t>
         </is>
       </c>
     </row>
@@ -694,22 +694,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jupiter72JUP</t>
+          <t>ether.fi90ETHFI</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>$0.1875</t>
+          <t>$0.5217</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.96%</t>
+          <t>7.49%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>$46,760,880</t>
+          <t>$50,332,903</t>
         </is>
       </c>
     </row>
@@ -719,22 +719,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ether.fi93ETHFI</t>
+          <t>Celestia99TIA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>$0.5115</t>
+          <t>$0.4135</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.80%</t>
+          <t>6.09%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>$43,732,238</t>
+          <t>$113,055,339</t>
         </is>
       </c>
     </row>
@@ -744,22 +744,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Venice Token98VVV</t>
+          <t>MemeCore22M</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>$9.14</t>
+          <t>$3.83</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7.48%</t>
+          <t>5.43%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>$18,638,618</t>
+          <t>$18,848,782</t>
         </is>
       </c>
     </row>
@@ -769,22 +769,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Virtuals Protocol84VIRTUAL</t>
+          <t>Kaspa59KAS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>$0.7756</t>
+          <t>$0.03565</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.18%</t>
+          <t>5.24%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>$131,878,689</t>
+          <t>$37,731,101</t>
         </is>
       </c>
     </row>
@@ -794,22 +794,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Aave44AAVE</t>
+          <t>Jupiter72JUP</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$116.54</t>
+          <t>$0.1865</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6.16%</t>
+          <t>4.61%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$539,567,157</t>
+          <t>$46,706,929</t>
         </is>
       </c>
     </row>
@@ -819,22 +819,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Arbitrum67ARB</t>
+          <t>Arbitrum66ARB</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$0.1308</t>
+          <t>$0.1331</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>5.92%</t>
+          <t>4.23%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$215,481,811</t>
+          <t>$212,722,783</t>
         </is>
       </c>
     </row>
@@ -844,22 +844,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Stellar17XLM</t>
+          <t>Quant61QNT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>$0.1745</t>
+          <t>$77.84</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5.44%</t>
+          <t>4.07%</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>$170,548,967</t>
+          <t>$13,719,793</t>
         </is>
       </c>
     </row>
@@ -869,22 +869,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sky40SKY</t>
+          <t>Stellar18XLM</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>$0.07877</t>
+          <t>$0.1734</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.90%</t>
+          <t>3.88%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>$18,685,520</t>
+          <t>$164,985,685</t>
         </is>
       </c>
     </row>
@@ -894,22 +894,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Monad90MON</t>
+          <t>Pi41PI</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>$0.03686</t>
+          <t>$0.1801</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4.89%</t>
+          <t>3.80%</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>$105,464,613</t>
+          <t>$32,143,316</t>
         </is>
       </c>
     </row>
@@ -919,22 +919,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pudgy Penguins85PENGU</t>
+          <t>Ethereum2ETH</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>$0.007981</t>
+          <t>$2,420.95</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>4.87%</t>
+          <t>3.33%</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>$191,776,762</t>
+          <t>$26,117,556,113</t>
         </is>
       </c>
     </row>
@@ -944,22 +944,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Quant62QNT</t>
+          <t>Virtuals Protocol83VIRTUAL</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>$78.54</t>
+          <t>$0.7669</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>4.69%</t>
+          <t>3.28%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>$12,856,050</t>
+          <t>$131,052,317</t>
         </is>
       </c>
     </row>
@@ -969,22 +969,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ethereum2ETH</t>
+          <t>GateToken64GT</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>$2,443.98</t>
+          <t>$7.31</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4.51%</t>
+          <t>3.10%</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>$25,375,917,895</t>
+          <t>$3,271,970</t>
         </is>
       </c>
     </row>
@@ -994,22 +994,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pi43PI</t>
+          <t>Sky42SKY</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>$0.1785</t>
+          <t>$0.07888</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>4.48%</t>
+          <t>3.07%</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>$32,751,842</t>
+          <t>$18,469,492</t>
         </is>
       </c>
     </row>
@@ -1019,22 +1019,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Mantle37MNT</t>
+          <t>Bitcoin1BTC</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>$0.6888</t>
+          <t>$77,201.15</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4.39%</t>
+          <t>3.05%</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>$51,533,552</t>
+          <t>$55,020,312,618</t>
         </is>
       </c>
     </row>
@@ -1044,22 +1044,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Pepe46PEPE</t>
+          <t>Nexo77NEXO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>$0.05405</t>
+          <t>$0.9279</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4.17%</t>
+          <t>2.93%</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>$753,685,072</t>
+          <t>$10,225,961</t>
         </is>
       </c>
     </row>
@@ -1069,22 +1069,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Bitcoin1BTC</t>
+          <t>Flare69FLR</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>$77,882.87</t>
+          <t>$0.008414</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>4.13%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>$53,195,207,080</t>
+          <t>$5,171,299</t>
         </is>
       </c>
     </row>
@@ -1094,22 +1094,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Uniswap39UNI</t>
+          <t>Aave44AAVE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>$3.51</t>
+          <t>$117.57</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>$264,299,084</t>
+          <t>$495,640,170</t>
         </is>
       </c>
     </row>
@@ -1119,22 +1119,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hedera28HBAR</t>
+          <t>Uniswap39UNI</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>$0.09227</t>
+          <t>$3.51</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3.98%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>$131,152,910</t>
+          <t>$267,609,589</t>
         </is>
       </c>
     </row>
@@ -1144,22 +1144,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Lido DAO101LDO</t>
+          <t>Tezos95XTZ</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>$0.4351</t>
+          <t>$0.3831</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3.97%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>$119,050,022</t>
+          <t>$15,496,640</t>
         </is>
       </c>
     </row>
@@ -1169,22 +1169,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Solana7SOL</t>
+          <t>XRP4XRP</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>$90.13</t>
+          <t>$1.48</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3.95%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>$7,643,314,897</t>
+          <t>$4,502,102,661</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Check Outlier in Lossers
</commit_message>
<xml_diff>
--- a/gainers.xlsx
+++ b/gainers.xlsx
@@ -444,22 +444,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>RaveDAO21RAVE</t>
+          <t>币安人生88币安人生</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>$20.91</t>
+          <t>$0.4744</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>27.46%</t>
+          <t>43.69%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>$274,717,861</t>
+          <t>$190,490,084</t>
         </is>
       </c>
     </row>
@@ -469,22 +469,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ethena54ENA</t>
+          <t>RaveDAO16RAVE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>$0.1282</t>
+          <t>$25.40</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>14.50%</t>
+          <t>40.87%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>$215,822,861</t>
+          <t>$339,060,748</t>
         </is>
       </c>
     </row>
@@ -494,22 +494,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Aerodrome Finance98AERO</t>
+          <t>MemeCore19M</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>$0.4397</t>
+          <t>$4.44</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>12.13%</t>
+          <t>15.59%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>$55,549,454</t>
+          <t>$26,253,827</t>
         </is>
       </c>
     </row>
@@ -519,22 +519,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DeXe55DEXE</t>
+          <t>DeXe54DEXE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>$12.29</t>
+          <t>$13.13</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>11.19%</t>
+          <t>12.23%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>$23,119,099</t>
+          <t>$32,136,735</t>
         </is>
       </c>
     </row>
@@ -544,22 +544,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>edgeX86EDGE</t>
+          <t>Ethena55ENA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>$1.35</t>
+          <t>$0.123</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.39%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$165,522,350</t>
+          <t>$269,728,278</t>
         </is>
       </c>
     </row>
@@ -569,22 +569,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Venice Token93VVV</t>
+          <t>edgeX87EDGE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>$9.34</t>
+          <t>$1.36</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>$21,763,205</t>
+          <t>$138,104,939</t>
         </is>
       </c>
     </row>
@@ -594,22 +594,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Morpho67MORPHO</t>
+          <t>Aerodrome Finance99AERO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>$1.95</t>
+          <t>$0.4336</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>8.58%</t>
+          <t>8.82%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>$28,951,998</t>
+          <t>$47,892,062</t>
         </is>
       </c>
     </row>
@@ -619,22 +619,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bittensor32TAO</t>
+          <t>Morpho65MORPHO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>$261.94</t>
+          <t>$1.94</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8.39%</t>
+          <t>8.45%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>$415,100,954</t>
+          <t>$29,223,876</t>
         </is>
       </c>
     </row>
@@ -644,22 +644,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>币安人生100币安人生</t>
+          <t>Pi40PI</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>$0.3666</t>
+          <t>$0.1849</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>7.67%</t>
+          <t>7.53%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>$143,972,828</t>
+          <t>$34,522,511</t>
         </is>
       </c>
     </row>
@@ -669,22 +669,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JUST79JST</t>
+          <t>JUST77JST</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>$0.06753</t>
+          <t>$0.07022</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>7.54%</t>
+          <t>7.41%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>$51,374,400</t>
+          <t>$42,730,397</t>
         </is>
       </c>
     </row>
@@ -694,22 +694,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ether.fi90ETHFI</t>
+          <t>Kaspa58KAS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>$0.5217</t>
+          <t>$0.03601</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.49%</t>
+          <t>6.81%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>$50,332,903</t>
+          <t>$37,960,750</t>
         </is>
       </c>
     </row>
@@ -719,22 +719,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Celestia99TIA</t>
+          <t>ether.fi92ETHFI</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>$0.4135</t>
+          <t>$0.5122</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>6.09%</t>
+          <t>6.35%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>$113,055,339</t>
+          <t>$48,026,902</t>
         </is>
       </c>
     </row>
@@ -744,22 +744,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MemeCore22M</t>
+          <t>Celestia100TIA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>$3.83</t>
+          <t>$0.4243</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>5.43%</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>$18,848,782</t>
+          <t>$105,508,407</t>
         </is>
       </c>
     </row>
@@ -769,22 +769,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Kaspa59KAS</t>
+          <t>Stellar18XLM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>$0.03565</t>
+          <t>$0.1745</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.24%</t>
+          <t>4.73%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>$37,731,101</t>
+          <t>$154,945,757</t>
         </is>
       </c>
     </row>
@@ -794,22 +794,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jupiter72JUP</t>
+          <t>Hyperliquid10HYPE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$0.1865</t>
+          <t>$45.20</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>4.61%</t>
+          <t>4.29%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$46,706,929</t>
+          <t>$316,982,812</t>
         </is>
       </c>
     </row>
@@ -819,22 +819,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Arbitrum66ARB</t>
+          <t>Virtuals Protocol84VIRTUAL</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$0.1331</t>
+          <t>$0.7508</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4.23%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$212,722,783</t>
+          <t>$122,329,630</t>
         </is>
       </c>
     </row>
@@ -844,22 +844,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Quant61QNT</t>
+          <t>Flare69FLR</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>$77.84</t>
+          <t>$0.00843</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.07%</t>
+          <t>3.45%</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>$13,719,793</t>
+          <t>$4,326,587</t>
         </is>
       </c>
     </row>
@@ -869,22 +869,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Stellar18XLM</t>
+          <t>Ethereum2ETH</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>$0.1734</t>
+          <t>$2,403.22</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.88%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>$164,985,685</t>
+          <t>$26,215,233,082</t>
         </is>
       </c>
     </row>
@@ -894,22 +894,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Pi41PI</t>
+          <t>Bitcoin1BTC</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>$0.1801</t>
+          <t>$77,004.25</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>3.80%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>$32,143,316</t>
+          <t>$52,601,505,491</t>
         </is>
       </c>
     </row>
@@ -919,22 +919,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ethereum2ETH</t>
+          <t>Mantle37MNT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>$2,420.95</t>
+          <t>$0.6825</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.33%</t>
+          <t>2.60%</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>$26,117,556,113</t>
+          <t>$46,082,085</t>
         </is>
       </c>
     </row>
@@ -944,22 +944,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Virtuals Protocol83VIRTUAL</t>
+          <t>XRP4XRP</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>$0.7669</t>
+          <t>$1.47</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3.28%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>$131,052,317</t>
+          <t>$3,990,928,952</t>
         </is>
       </c>
     </row>
@@ -969,22 +969,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GateToken64GT</t>
+          <t>Uniswap39UNI</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>$7.31</t>
+          <t>$3.44</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.10%</t>
+          <t>2.45%</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>$3,271,970</t>
+          <t>$247,690,769</t>
         </is>
       </c>
     </row>
@@ -994,22 +994,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sky42SKY</t>
+          <t>Midnight76NIGHT</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>$0.07888</t>
+          <t>$0.0369</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3.07%</t>
+          <t>2.44%</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>$18,469,492</t>
+          <t>$24,008,932</t>
         </is>
       </c>
     </row>
@@ -1019,22 +1019,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Bitcoin1BTC</t>
+          <t>Polkadot38DOT</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>$77,201.15</t>
+          <t>$1.33</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3.05%</t>
+          <t>2.42%</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>$55,020,312,618</t>
+          <t>$251,643,657</t>
         </is>
       </c>
     </row>
@@ -1044,22 +1044,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nexo77NEXO</t>
+          <t>Monad95MON</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>$0.9279</t>
+          <t>$0.03456</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2.93%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>$10,225,961</t>
+          <t>$101,156,616</t>
         </is>
       </c>
     </row>
@@ -1069,22 +1069,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Flare69FLR</t>
+          <t>Ondo52ONDO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>$0.008414</t>
+          <t>$0.2694</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2.82%</t>
+          <t>1.82%</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>$5,171,299</t>
+          <t>$90,290,615</t>
         </is>
       </c>
     </row>
@@ -1094,22 +1094,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Aave44AAVE</t>
+          <t>BNB5BNB</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>$117.57</t>
+          <t>$640.79</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>1.80%</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>$495,640,170</t>
+          <t>$2,031,349,352</t>
         </is>
       </c>
     </row>
@@ -1119,22 +1119,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Uniswap39UNI</t>
+          <t>Sky43SKY</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>$3.51</t>
+          <t>$0.07777</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>$267,609,589</t>
+          <t>$18,060,108</t>
         </is>
       </c>
     </row>
@@ -1144,22 +1144,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Tezos95XTZ</t>
+          <t>Venice Token98VVV</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>$0.3831</t>
+          <t>$8.78</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>1.54%</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>$15,496,640</t>
+          <t>$23,602,987</t>
         </is>
       </c>
     </row>
@@ -1169,22 +1169,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>XRP4XRP</t>
+          <t>Cosmos63ATOM</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>$1.48</t>
+          <t>$1.84</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>1.53%</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>$4,502,102,661</t>
+          <t>$66,273,919</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: handling outlier gainners
</commit_message>
<xml_diff>
--- a/gainers.xlsx
+++ b/gainers.xlsx
@@ -444,22 +444,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>币安人生88币安人生</t>
+          <t>币安人生85币安人生</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>$0.4744</t>
+          <t>$0.5238</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>43.69%</t>
+          <t>58.05%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>$190,490,084</t>
+          <t>$207,418,787</t>
         </is>
       </c>
     </row>
@@ -469,22 +469,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RaveDAO16RAVE</t>
+          <t>MemeCore18M</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>$25.40</t>
+          <t>$4.46</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>40.87%</t>
+          <t>17.65%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>$339,060,748</t>
+          <t>$27,099,072</t>
         </is>
       </c>
     </row>
@@ -494,22 +494,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MemeCore19M</t>
+          <t>Ethena55ENA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>$4.44</t>
+          <t>$0.1229</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>15.59%</t>
+          <t>12.09%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>$26,253,827</t>
+          <t>$272,105,922</t>
         </is>
       </c>
     </row>
@@ -519,22 +519,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DeXe54DEXE</t>
+          <t>edgeX88EDGE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>$13.13</t>
+          <t>$1.39</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>12.23%</t>
+          <t>10.55%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>$32,136,735</t>
+          <t>$135,394,215</t>
         </is>
       </c>
     </row>
@@ -544,22 +544,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ethena55ENA</t>
+          <t>DeXe54DEXE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>$0.123</t>
+          <t>$13.13</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$269,728,278</t>
+          <t>$31,778,918</t>
         </is>
       </c>
     </row>
@@ -569,22 +569,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>edgeX87EDGE</t>
+          <t>Aerodrome Finance99AERO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>$1.36</t>
+          <t>$0.4335</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>8.37%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>$138,104,939</t>
+          <t>$48,021,028</t>
         </is>
       </c>
     </row>
@@ -594,22 +594,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Aerodrome Finance99AERO</t>
+          <t>Morpho65MORPHO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>$0.4336</t>
+          <t>$1.94</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>8.82%</t>
+          <t>8.12%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>$47,892,062</t>
+          <t>$29,400,080</t>
         </is>
       </c>
     </row>
@@ -619,22 +619,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Morpho65MORPHO</t>
+          <t>ether.fi93ETHFI</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>$1.94</t>
+          <t>$0.5159</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8.45%</t>
+          <t>7.61%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>$29,223,876</t>
+          <t>$48,617,051</t>
         </is>
       </c>
     </row>
@@ -649,17 +649,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>$0.1849</t>
+          <t>$0.1848</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>7.53%</t>
+          <t>6.95%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>$34,522,511</t>
+          <t>$34,679,003</t>
         </is>
       </c>
     </row>
@@ -669,22 +669,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JUST77JST</t>
+          <t>Celestia100TIA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>$0.07022</t>
+          <t>$0.4213</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>7.41%</t>
+          <t>6.42%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>$42,730,397</t>
+          <t>$105,729,098</t>
         </is>
       </c>
     </row>
@@ -694,22 +694,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Kaspa58KAS</t>
+          <t>JUST77JST</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>$0.03601</t>
+          <t>$0.06962</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>6.81%</t>
+          <t>5.70%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>$37,960,750</t>
+          <t>$41,979,044</t>
         </is>
       </c>
     </row>
@@ -719,22 +719,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ether.fi92ETHFI</t>
+          <t>Kaspa58KAS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>$0.5122</t>
+          <t>$0.03577</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>6.35%</t>
+          <t>5.60%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>$48,026,902</t>
+          <t>$38,396,401</t>
         </is>
       </c>
     </row>
@@ -744,22 +744,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Celestia100TIA</t>
+          <t>Stellar19XLM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>$0.4243</t>
+          <t>$0.1742</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>4.93%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>$105,508,407</t>
+          <t>$162,401,338</t>
         </is>
       </c>
     </row>
@@ -769,22 +769,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Stellar18XLM</t>
+          <t>Virtuals Protocol86VIRTUAL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>$0.1745</t>
+          <t>$0.7512</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4.73%</t>
+          <t>3.63%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>$154,945,757</t>
+          <t>$122,772,801</t>
         </is>
       </c>
     </row>
@@ -799,17 +799,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$45.20</t>
+          <t>$44.97</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>4.29%</t>
+          <t>3.12%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$316,982,812</t>
+          <t>$320,196,555</t>
         </is>
       </c>
     </row>
@@ -819,22 +819,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Virtuals Protocol84VIRTUAL</t>
+          <t>Ethereum2ETH</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$0.7508</t>
+          <t>$2,405.35</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.10%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$122,329,630</t>
+          <t>$26,536,344,318</t>
         </is>
       </c>
     </row>
@@ -844,22 +844,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Flare69FLR</t>
+          <t>Bitcoin1BTC</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>$0.00843</t>
+          <t>$77,047.54</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.45%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>$4,326,587</t>
+          <t>$52,917,237,070</t>
         </is>
       </c>
     </row>
@@ -869,22 +869,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ethereum2ETH</t>
+          <t>Flare69FLR</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>$2,403.22</t>
+          <t>$0.00844</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>$26,215,233,082</t>
+          <t>$4,316,922</t>
         </is>
       </c>
     </row>
@@ -894,22 +894,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bitcoin1BTC</t>
+          <t>Uniswap39UNI</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>$77,004.25</t>
+          <t>$3.46</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>3.17%</t>
+          <t>2.90%</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>$52,601,505,491</t>
+          <t>$249,145,848</t>
         </is>
       </c>
     </row>
@@ -924,17 +924,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>$0.6825</t>
+          <t>$0.6816</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.60%</t>
+          <t>2.64%</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>$46,082,085</t>
+          <t>$45,943,311</t>
         </is>
       </c>
     </row>
@@ -954,12 +954,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>$3,990,928,952</t>
+          <t>$3,989,123,232</t>
         </is>
       </c>
     </row>
@@ -969,22 +969,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Uniswap39UNI</t>
+          <t>BNB5BNB</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>$3.44</t>
+          <t>$643.53</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.45%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>$247,690,769</t>
+          <t>$2,037,873,566</t>
         </is>
       </c>
     </row>
@@ -994,22 +994,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Midnight76NIGHT</t>
+          <t>Chiliz90CHZ</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>$0.0369</t>
+          <t>$0.04215</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2.44%</t>
+          <t>2.00%</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>$24,008,932</t>
+          <t>$65,052,650</t>
         </is>
       </c>
     </row>
@@ -1024,17 +1024,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>$1.33</t>
+          <t>$1.32</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2.42%</t>
+          <t>1.93%</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>$251,643,657</t>
+          <t>$249,705,287</t>
         </is>
       </c>
     </row>
@@ -1044,22 +1044,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Monad95MON</t>
+          <t>Arbitrum67ARB</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>$0.03456</t>
+          <t>$0.1305</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2.30%</t>
+          <t>1.76%</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>$101,156,616</t>
+          <t>$179,898,261</t>
         </is>
       </c>
     </row>
@@ -1069,22 +1069,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ondo52ONDO</t>
+          <t>GateToken64GT</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>$0.2694</t>
+          <t>$7.35</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1.82%</t>
+          <t>1.62%</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>$90,290,615</t>
+          <t>$3,122,006</t>
         </is>
       </c>
     </row>
@@ -1094,22 +1094,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BNB5BNB</t>
+          <t>Cosmos63ATOM</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>$640.79</t>
+          <t>$1.83</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1.80%</t>
+          <t>1.59%</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>$2,031,349,352</t>
+          <t>$66,286,920</t>
         </is>
       </c>
     </row>
@@ -1119,22 +1119,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sky43SKY</t>
+          <t>Monad96MON</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>$0.07777</t>
+          <t>$0.03433</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>1.55%</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>$18,060,108</t>
+          <t>$101,358,789</t>
         </is>
       </c>
     </row>
@@ -1144,22 +1144,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Venice Token98VVV</t>
+          <t>Bittensor32TAO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>$8.78</t>
+          <t>$252.36</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1.54%</t>
+          <t>1.50%</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>$23,602,987</t>
+          <t>$352,750,050</t>
         </is>
       </c>
     </row>
@@ -1169,22 +1169,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cosmos63ATOM</t>
+          <t>Ondo52ONDO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>$1.84</t>
+          <t>$0.2694</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1.53%</t>
+          <t>1.50%</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>$66,273,919</t>
+          <t>$89,334,731</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add visualitation pie chart
</commit_message>
<xml_diff>
--- a/gainers.xlsx
+++ b/gainers.xlsx
@@ -441,660 +441,660 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>edgeX83EDGE</t>
+          <t>RaveDAO89RAVE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>$1.35</t>
+          <t>$2.09</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>16.24%</t>
+          <t>259.37%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>$50,504,723</t>
+          <t>$583,479,523</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>币安人生88币安人生</t>
+          <t>币安人生86币安人生</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>$0.4397</t>
+          <t>$0.4712</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>11.36%</t>
+          <t>16.54%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>$134,452,521</t>
+          <t>$101,851,514</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>siren80SIREN</t>
+          <t>Pudgy Penguins84PENGU</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>$0.7056</t>
+          <t>$0.007551</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>9.98%</t>
+          <t>6.38%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>$22,413,558</t>
+          <t>$130,796,596</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chiliz86CHZ</t>
+          <t>Chiliz83CHZ</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$0.04344</t>
+          <t>$0.04611</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.47%</t>
+          <t>5.26%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>$95,299,665</t>
+          <t>$186,473,288</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sky39SKY</t>
+          <t>Toncoin29TON</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$0.07922</t>
+          <t>$1.36</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.43%</t>
+          <t>4.19%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>$15,942,209</t>
+          <t>$168,158,164</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Canton16CC</t>
+          <t>Venice Token91VVV</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$0.152</t>
+          <t>$9.38</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2.88%</t>
+          <t>4.10%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>$13,241,816</t>
+          <t>$18,963,374</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JUST70JST</t>
+          <t>Canton16CC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>$0.07391</t>
+          <t>$0.1568</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2.59%</t>
+          <t>4.01%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>$34,025,937</t>
+          <t>$20,902,642</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Polygon (prev. MATIC)56POL</t>
+          <t>MemeCore21M</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>$0.09032</t>
+          <t>$3.37</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.47%</t>
+          <t>3.80%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>$58,278,294</t>
+          <t>$24,938,158</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Pudgy Penguins85PENGU</t>
+          <t>Monad98MON</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>$0.007224</t>
+          <t>$0.03113</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.27%</t>
+          <t>3.54%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>$112,948,067</t>
+          <t>$80,591,812</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bonk79BONK</t>
+          <t>Stellar17XLM</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>$0.056059</t>
+          <t>$0.1743</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.17%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>$67,881,564</t>
+          <t>$123,974,176</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GateToken63GT</t>
+          <t>LayerZero79ZRO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>$7.21</t>
+          <t>$1.67</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.04%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>$2,964,280</t>
+          <t>$115,347,776</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DeXe51DEXE</t>
+          <t>Polygon (prev. MATIC)55POL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>$15.17</t>
+          <t>$0.09196</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.93%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>$41,219,530</t>
+          <t>$70,282,517</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Arbitrum65ARB</t>
+          <t>Kaspa57KAS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>$0.1262</t>
+          <t>$0.03536</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.81%</t>
+          <t>2.58%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>$91,572,250</t>
+          <t>$25,870,484</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MemeCore21M</t>
+          <t>World Liberty Financial33WLFI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>$3.49</t>
+          <t>$0.07938</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.81%</t>
+          <t>2.35%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>$27,661,077</t>
+          <t>$52,357,848</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bitget Token49BGB</t>
+          <t>Sky39SKY</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$1.88</t>
+          <t>$0.07918</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.72%</t>
+          <t>2.31%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$62,812,583</t>
+          <t>$24,733,120</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aster43ASTER</t>
+          <t>GateToken63GT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$0.6785</t>
+          <t>$7.28</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.54%</t>
+          <t>2.10%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$157,452,159</t>
+          <t>$2,991,028</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hedera26HBAR</t>
+          <t>JUST70JST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>$0.08875</t>
+          <t>$0.07512</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>1.97%</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>$105,232,978</t>
+          <t>$28,189,908</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NEAR Protocol42NEAR</t>
+          <t>UNUS SED LEO11LEO</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>$1.34</t>
+          <t>$10.34</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>1.97%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>$221,395,588</t>
+          <t>$1,578,029</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Worldcoin62WLD</t>
+          <t>Sei96SEI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>$0.2618</t>
+          <t>$0.05593</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>1.77%</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>$132,844,001</t>
+          <t>$25,256,969</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ethereum Classic50ETC</t>
+          <t>Avalanche24AVAX</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>$8.38</t>
+          <t>$9.31</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.52%</t>
+          <t>1.76%</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>$43,372,951</t>
+          <t>$329,416,426</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>KuCoin Token53KCS</t>
+          <t>Render58RENDER</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>$8.51</t>
+          <t>$1.79</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.46%</t>
+          <t>1.72%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>$19,736,205</t>
+          <t>$70,677,644</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BNB5BNB</t>
+          <t>Cronos30CRO</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>$623.77</t>
+          <t>$0.07029</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.39%</t>
+          <t>1.71%</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>$1,503,958,909</t>
+          <t>$7,079,735</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dash89DASH</t>
+          <t>edgeX87EDGE</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>$34.07</t>
+          <t>$1.33</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.35%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>$65,562,277</t>
+          <t>$54,199,617</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aave46AAVE</t>
+          <t>Aerodrome Finance99AERO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>$91.54</t>
+          <t>$0.3835</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>$692,049,895</t>
+          <t>$19,962,317</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Render58RENDER</t>
+          <t>Bonk78BONK</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>$1.77</t>
+          <t>$0.056111</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>1.57%</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>$72,882,252</t>
+          <t>$54,329,361</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>UNUS SED LEO11LEO</t>
+          <t>Pump.fun72PUMP</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>$10.17</t>
+          <t>$0.001831</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>$589,305</t>
+          <t>$42,705,201</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Virtuals Protocol87VIRTUAL</t>
+          <t>Mantle37MNT</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>$0.6861</t>
+          <t>$0.6298</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.25%</t>
+          <t>1.46%</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>$92,122,276</t>
+          <t>$1,392,856,815</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Venice Token92VVV</t>
+          <t>Aave46AAVE</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>$9.07</t>
+          <t>$94.66</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.15%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>$19,563,284</t>
+          <t>$619,856,384</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Stellar17XLM</t>
+          <t>Bitcoin1BTC</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>$0.1684</t>
+          <t>$75,717.14</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>$108,902,468</t>
+          <t>$38,154,063,324</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dogecoin9DOGE</t>
+          <t>Zcash19ZEC</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>$0.09426</t>
+          <t>$317.09</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>1.44%</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>$1,910,002,040</t>
+          <t>$362,437,127</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add chart top volume
</commit_message>
<xml_diff>
--- a/gainers.xlsx
+++ b/gainers.xlsx
@@ -441,88 +441,88 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RaveDAO89RAVE</t>
+          <t>RaveDAO88RAVE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>$2.09</t>
+          <t>$1.88</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>259.37%</t>
+          <t>254.63%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>$583,479,523</t>
+          <t>$696,161,103</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>币安人生86币安人生</t>
+          <t>Chiliz87CHZ</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>$0.4712</t>
+          <t>$0.04631</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>16.54%</t>
+          <t>7.31%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>$101,851,514</t>
+          <t>$178,110,586</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pudgy Penguins84PENGU</t>
+          <t>币安人生84币安人生</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>$0.007551</t>
+          <t>$0.4847</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.38%</t>
+          <t>6.93%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>$130,796,596</t>
+          <t>$99,938,507</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chiliz83CHZ</t>
+          <t>Monad97MON</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$0.04611</t>
+          <t>$0.03244</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.26%</t>
+          <t>6.83%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>$186,473,288</t>
+          <t>$81,929,277</t>
         </is>
       </c>
     </row>
@@ -534,567 +534,567 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$1.36</t>
+          <t>$1.38</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>6.70%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>$168,158,164</t>
+          <t>$183,687,570</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Venice Token91VVV</t>
+          <t>Stellar16XLM</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$9.38</t>
+          <t>$0.1795</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>4.10%</t>
+          <t>6.33%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>$18,963,374</t>
+          <t>$132,118,027</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Canton16CC</t>
+          <t>Pudgy Penguins86PENGU</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>$0.1568</t>
+          <t>$0.007645</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4.01%</t>
+          <t>5.79%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>$20,902,642</t>
+          <t>$138,363,380</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MemeCore21M</t>
+          <t>LayerZero79ZRO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>$3.37</t>
+          <t>$1.65</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3.80%</t>
+          <t>5.57%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>$24,938,158</t>
+          <t>$106,946,583</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Monad98MON</t>
+          <t>JUST70JST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>$0.03113</t>
+          <t>$0.07724</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>3.54%</t>
+          <t>5.38%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>$80,591,812</t>
+          <t>$28,666,633</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Stellar17XLM</t>
+          <t>Mantle37MNT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>$0.1743</t>
+          <t>$0.6434</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>4.85%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>$123,974,176</t>
+          <t>$1,311,857,853</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LayerZero79ZRO</t>
+          <t>edgeX83EDGE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>$1.67</t>
+          <t>$1.39</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>$115,347,776</t>
+          <t>$52,707,256</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Polygon (prev. MATIC)55POL</t>
+          <t>Zcash19ZEC</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>$0.09196</t>
+          <t>$318.16</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>3.43%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>$70,282,517</t>
+          <t>$397,947,861</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kaspa57KAS</t>
+          <t>Polygon (prev. MATIC)55POL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>$0.03536</t>
+          <t>$0.0927</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.58%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>$25,870,484</t>
+          <t>$7,909,370,571</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>World Liberty Financial33WLFI</t>
+          <t>Venice Token92VVV</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>$0.07938</t>
+          <t>$9.35</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.35%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>$52,357,848</t>
+          <t>$17,271,674</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sky39SKY</t>
+          <t>NEAR Protocol40NEAR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$0.07918</t>
+          <t>$1.38</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2.31%</t>
+          <t>2.76%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$24,733,120</t>
+          <t>$177,896,111</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GateToken63GT</t>
+          <t>Kaspa57KAS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$7.28</t>
+          <t>$0.03512</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2.10%</t>
+          <t>2.74%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$2,991,028</t>
+          <t>$25,171,206</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>JUST70JST</t>
+          <t>Sky39SKY</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>$0.07512</t>
+          <t>$0.08006</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.97%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>$28,189,908</t>
+          <t>$24,590,767</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>UNUS SED LEO11LEO</t>
+          <t>Morpho64MORPHO</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>$10.34</t>
+          <t>$1.98</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.97%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>$1,578,029</t>
+          <t>$14,648,721</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sei96SEI</t>
+          <t>Monero15XMR</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>$0.05593</t>
+          <t>$361.96</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.77%</t>
+          <t>2.33%</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>$25,256,969</t>
+          <t>$116,114,636</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Avalanche24AVAX</t>
+          <t>Artificial Superintelligence Alliance85FET</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>$9.31</t>
+          <t>$0.2137</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.76%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>$329,416,426</t>
+          <t>$138,995,094</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Render58RENDER</t>
+          <t>Hedera25HBAR</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>$1.79</t>
+          <t>$0.09065</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.72%</t>
+          <t>2.29%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>$70,677,644</t>
+          <t>$119,901,811</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cronos30CRO</t>
+          <t>Nexo76NEXO</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>$0.07029</t>
+          <t>$0.902</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.71%</t>
+          <t>2.26%</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>$7,079,735</t>
+          <t>$8,456,724</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>edgeX87EDGE</t>
+          <t>World Liberty Financial33WLFI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>$1.33</t>
+          <t>$0.07909</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>$54,199,617</t>
+          <t>$49,926,113</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aerodrome Finance99AERO</t>
+          <t>Ondo51ONDO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>$0.3835</t>
+          <t>$0.258</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>$19,962,317</t>
+          <t>$83,505,013</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Bonk78BONK</t>
+          <t>Quant61QNT</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>$0.056111</t>
+          <t>$74.78</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1.57%</t>
+          <t>2.08%</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>$54,329,361</t>
+          <t>$8,038,684</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pump.fun72PUMP</t>
+          <t>Render58RENDER</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>$0.001831</t>
+          <t>$1.80</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>$42,705,201</t>
+          <t>$69,366,863</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mantle37MNT</t>
+          <t>Pump.fun72PUMP</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>$0.6298</t>
+          <t>$0.001843</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1.46%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>$1,392,856,815</t>
+          <t>$48,834,709</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Aave46AAVE</t>
+          <t>Sei96SEI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>$94.66</t>
+          <t>$0.05614</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>2.02%</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>$619,856,384</t>
+          <t>$24,161,053</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Bitcoin1BTC</t>
+          <t>XRP4XRP</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>$75,717.14</t>
+          <t>$1.44</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>1.88%</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>$38,154,063,324</t>
+          <t>$2,640,128,286</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Zcash19ZEC</t>
+          <t>Polkadot36DOT</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>$317.09</t>
+          <t>$1.28</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1.44%</t>
+          <t>1.83%</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>$362,437,127</t>
+          <t>$18,281,411,031</t>
         </is>
       </c>
     </row>

</xml_diff>